<commit_message>
updates on outreach tab
</commit_message>
<xml_diff>
--- a/excels/outreach_activity.xlsx
+++ b/excels/outreach_activity.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DEADE5C-40BF-4F95-AFC0-EE3FCAC82FE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC97358F-ECC4-4CE4-862E-AF144A6F7B17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="faculty_papers_Images" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="51">
   <si>
     <t>Title</t>
   </si>
@@ -80,6 +80,105 @@
   </si>
   <si>
     <t>02-05-2026</t>
+  </si>
+  <si>
+    <t>02-05-2027</t>
+  </si>
+  <si>
+    <t>02-05-2028</t>
+  </si>
+  <si>
+    <t>02-05-2029</t>
+  </si>
+  <si>
+    <t>02-05-2030</t>
+  </si>
+  <si>
+    <t>02-05-2031</t>
+  </si>
+  <si>
+    <t>02-05-2032</t>
+  </si>
+  <si>
+    <t>02-05-2033</t>
+  </si>
+  <si>
+    <t>02-05-2034</t>
+  </si>
+  <si>
+    <t>02-05-2035</t>
+  </si>
+  <si>
+    <t>02-05-2036</t>
+  </si>
+  <si>
+    <t>02-05-2037</t>
+  </si>
+  <si>
+    <t>02-05-2038</t>
+  </si>
+  <si>
+    <t>02-05-2039</t>
+  </si>
+  <si>
+    <t>02-05-2040</t>
+  </si>
+  <si>
+    <t>02-05-2041</t>
+  </si>
+  <si>
+    <t>02-05-2042</t>
+  </si>
+  <si>
+    <t>01-05-2027</t>
+  </si>
+  <si>
+    <t>01-05-2028</t>
+  </si>
+  <si>
+    <t>01-05-2029</t>
+  </si>
+  <si>
+    <t>01-05-2030</t>
+  </si>
+  <si>
+    <t>01-05-2031</t>
+  </si>
+  <si>
+    <t>01-05-2032</t>
+  </si>
+  <si>
+    <t>01-05-2033</t>
+  </si>
+  <si>
+    <t>01-05-2034</t>
+  </si>
+  <si>
+    <t>01-05-2035</t>
+  </si>
+  <si>
+    <t>01-05-2036</t>
+  </si>
+  <si>
+    <t>01-05-2037</t>
+  </si>
+  <si>
+    <t>01-05-2038</t>
+  </si>
+  <si>
+    <t>01-05-2039</t>
+  </si>
+  <si>
+    <t>01-05-2040</t>
+  </si>
+  <si>
+    <t>01-05-2041</t>
+  </si>
+  <si>
+    <t>01-05-2042</t>
+  </si>
+  <si>
+    <t>01-05-2043</t>
   </si>
 </sst>
 </file>
@@ -463,7 +562,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{761EB44B-A036-4E63-8CD7-0F5156F6EC40}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -493,6 +592,270 @@
         <v>15</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B28" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B34" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B35" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
outreach activity data update
</commit_message>
<xml_diff>
--- a/excels/outreach_activity.xlsx
+++ b/excels/outreach_activity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E5C48E-7244-4BBB-BEF3-ADBA826E3946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBFCB06E-4E7C-4EE8-BF02-4505F9F1429F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="faculty_papers_Images" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="104">
   <si>
     <t>Title</t>
   </si>
@@ -34,15 +34,6 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Description 1</t>
-  </si>
-  <si>
-    <t>Description 2</t>
-  </si>
-  <si>
-    <t>Description 3</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
@@ -175,132 +166,45 @@
     <t>link3</t>
   </si>
   <si>
-    <t>Description 4</t>
-  </si>
-  <si>
     <t>link4</t>
   </si>
   <si>
-    <t>Description 5</t>
-  </si>
-  <si>
     <t>link5</t>
   </si>
   <si>
-    <t>Description 6</t>
-  </si>
-  <si>
     <t>link6</t>
   </si>
   <si>
-    <t>Description 7</t>
-  </si>
-  <si>
     <t>link7</t>
   </si>
   <si>
-    <t>Description 8</t>
-  </si>
-  <si>
     <t>link8</t>
   </si>
   <si>
-    <t>Description 9</t>
-  </si>
-  <si>
     <t>link9</t>
   </si>
   <si>
-    <t>Description 10</t>
-  </si>
-  <si>
     <t>link10</t>
   </si>
   <si>
-    <t>Description 11</t>
-  </si>
-  <si>
     <t>link11</t>
   </si>
   <si>
-    <t>Description 12</t>
-  </si>
-  <si>
     <t>link12</t>
   </si>
   <si>
-    <t>Description 13</t>
-  </si>
-  <si>
     <t>link13</t>
   </si>
   <si>
-    <t>Description 14</t>
-  </si>
-  <si>
     <t>link14</t>
   </si>
   <si>
-    <t>Description 15</t>
-  </si>
-  <si>
     <t>link15</t>
   </si>
   <si>
-    <t>Description 16</t>
-  </si>
-  <si>
     <t>link16</t>
   </si>
   <si>
-    <t>Title1</t>
-  </si>
-  <si>
-    <t>Title2</t>
-  </si>
-  <si>
-    <t>Title3</t>
-  </si>
-  <si>
-    <t>Title4</t>
-  </si>
-  <si>
-    <t>Title5</t>
-  </si>
-  <si>
-    <t>Title6</t>
-  </si>
-  <si>
-    <t>Title7</t>
-  </si>
-  <si>
-    <t>Title8</t>
-  </si>
-  <si>
-    <t>Title9</t>
-  </si>
-  <si>
-    <t>Title10</t>
-  </si>
-  <si>
-    <t>Title11</t>
-  </si>
-  <si>
-    <t>Title12</t>
-  </si>
-  <si>
-    <t>Title13</t>
-  </si>
-  <si>
-    <t>Title14</t>
-  </si>
-  <si>
-    <t>Title15</t>
-  </si>
-  <si>
-    <t>Title16</t>
-  </si>
-  <si>
     <t>icon 1</t>
   </si>
   <si>
@@ -347,6 +251,93 @@
   </si>
   <si>
     <t>icon 16</t>
+  </si>
+  <si>
+    <t>Nodal Officer, Jan Jatiya Gaurav Diwas (JJGD) (Continuing from October, 2025)</t>
+  </si>
+  <si>
+    <t>Chairperson, Constitution of the Scrap Value Assessment Committee (Continuing from September, 2025)</t>
+  </si>
+  <si>
+    <t>Member, Constitution of Committee for Special Campaign for Disposal of Pending Matter (SCDPM 5.0) (Continuing from September, 2025)</t>
+  </si>
+  <si>
+    <t>Member, Committee for Organizing Institute Foundation Day Celebrations (September, 2025 - October, 2025)</t>
+  </si>
+  <si>
+    <t>Member, Committee for Swachatha Pakhwada-2025 (Continuing from September, 2025)</t>
+  </si>
+  <si>
+    <t>Chairman, Center for Diversity and Inclusivity (May, 2025 - May, 2026)</t>
+  </si>
+  <si>
+    <t>Member, Institute Affair Committee (Continuing from May, 2025)</t>
+  </si>
+  <si>
+    <t>Member, CCMT/CCMN/JoSAA 2025 Admissions (Continuing from March, 2025)</t>
+  </si>
+  <si>
+    <t>Member, Institute Infrastructure and Sustainability (Continuing from February, 2025)</t>
+  </si>
+  <si>
+    <t>Professor In Charge (Kalam Guest House, Kadam Guest House-Hyderabad and Outreach Centre) (Continuing from January, 2025)</t>
+  </si>
+  <si>
+    <t>Chairman, Food Quality in Kalam Guest House (Continuing from January, 2025)</t>
+  </si>
+  <si>
+    <t>Professor-In-Charge, Guest House (Continuing from January, 2025)</t>
+  </si>
+  <si>
+    <t>Member, Alumni Relations and Endowment Chair and Scholarship (Continuing from November, 2024)</t>
+  </si>
+  <si>
+    <t>Member, Committee for Swachatha Pakhwada-2024 (Continuing from August, 2024)</t>
+  </si>
+  <si>
+    <t>Chairperson, Campus Hygiene Committee (Continuing from July, 2024)</t>
+  </si>
+  <si>
+    <t>Head, Transportation Division and Program Coordinator (Continuing from July, 2024)</t>
+  </si>
+  <si>
+    <t>Professor In-Charge, Outreach Center and Staff Quarters Maintenance (Continuing from July, 2024)</t>
+  </si>
+  <si>
+    <t>Senate Nominee, Institute Standing Disciplinary Committee (Continuing from July, 2024)</t>
+  </si>
+  <si>
+    <t>FIC of Transportation Division Consultancy Works (August, 2022 - December, 2023)</t>
+  </si>
+  <si>
+    <t>Faculty Advisor of III B.Tech Civil Engineering (August, 2020 - August, 2022)</t>
+  </si>
+  <si>
+    <t>Warden of NITW Ganga Mess (July, 2018 - July, 2020)</t>
+  </si>
+  <si>
+    <t>Deputy Chief Warden (July, 2018 - July, 2020)</t>
+  </si>
+  <si>
+    <t>Member of Hostel Purchase Committee (July, 2018 - July, 2020)</t>
+  </si>
+  <si>
+    <t>Warden of NITW Hostels Sanitary Section (July, 2018 - July, 2020)</t>
+  </si>
+  <si>
+    <t>Member of Anti-Ragging Committee (July, 2016 - July, 2018)</t>
+  </si>
+  <si>
+    <t>Warden of NITW 1K Hall of Residence (March, 2014 - March, 2016)</t>
+  </si>
+  <si>
+    <t>FIC Transportation Division Library (January, 2014 - January, 2018)</t>
+  </si>
+  <si>
+    <t>FIC Pavement Evaluation Laboratory (September, 2013 - August, 2018)</t>
+  </si>
+  <si>
+    <t>FIC Pavement Materials Laboratory (September, 2013 - August, 2022)</t>
   </si>
 </sst>
 </file>
@@ -671,7 +662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
@@ -687,234 +678,251 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>75</v>
       </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
       <c r="C2" t="s">
-        <v>91</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>76</v>
       </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
       <c r="C3" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="D3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>77</v>
       </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
       <c r="C4" t="s">
-        <v>93</v>
+        <v>61</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>78</v>
       </c>
-      <c r="B5" t="s">
-        <v>49</v>
-      </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>62</v>
       </c>
       <c r="D5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>79</v>
       </c>
-      <c r="B6" t="s">
-        <v>51</v>
-      </c>
       <c r="C6" t="s">
-        <v>95</v>
+        <v>63</v>
       </c>
       <c r="D6" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>80</v>
       </c>
-      <c r="B7" t="s">
-        <v>53</v>
-      </c>
       <c r="C7" t="s">
-        <v>96</v>
+        <v>64</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>81</v>
       </c>
-      <c r="B8" t="s">
-        <v>55</v>
-      </c>
       <c r="C8" t="s">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="D8" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>82</v>
       </c>
-      <c r="B9" t="s">
-        <v>57</v>
-      </c>
       <c r="C9" t="s">
-        <v>98</v>
+        <v>66</v>
       </c>
       <c r="D9" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>83</v>
       </c>
-      <c r="B10" t="s">
-        <v>59</v>
-      </c>
       <c r="C10" t="s">
-        <v>99</v>
+        <v>67</v>
       </c>
       <c r="D10" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>84</v>
       </c>
-      <c r="B11" t="s">
-        <v>61</v>
-      </c>
       <c r="C11" t="s">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="D11" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>85</v>
       </c>
-      <c r="B12" t="s">
-        <v>63</v>
-      </c>
       <c r="C12" t="s">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="D12" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>86</v>
       </c>
-      <c r="B13" t="s">
-        <v>65</v>
-      </c>
       <c r="C13" t="s">
-        <v>102</v>
+        <v>70</v>
       </c>
       <c r="D13" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>87</v>
       </c>
-      <c r="B14" t="s">
-        <v>67</v>
-      </c>
       <c r="C14" t="s">
-        <v>103</v>
+        <v>71</v>
       </c>
       <c r="D14" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>88</v>
       </c>
-      <c r="B15" t="s">
-        <v>69</v>
-      </c>
       <c r="C15" t="s">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="D15" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>89</v>
       </c>
-      <c r="B16" t="s">
-        <v>71</v>
-      </c>
       <c r="C16" t="s">
-        <v>105</v>
+        <v>73</v>
       </c>
       <c r="D16" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>90</v>
       </c>
-      <c r="B17" t="s">
-        <v>73</v>
-      </c>
       <c r="C17" t="s">
-        <v>106</v>
+        <v>74</v>
       </c>
       <c r="D17" t="s">
-        <v>74</v>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -933,290 +941,290 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B14" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B18" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B19" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B20" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B22" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B23" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B25" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B28" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B29" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B30" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B31" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B32" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B33" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B34" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B35" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B36" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>